<commit_message>
not update after socket
</commit_message>
<xml_diff>
--- a/configs/Skill.xlsx
+++ b/configs/Skill.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28827"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yatyr\workspace\gvbasic-mir-remaster\configs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{009571B3-EC72-4378-9B2B-25D706B2584E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8EB1732C-9118-4793-850E-69C926777FDD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19110" yWindow="0" windowWidth="19380" windowHeight="20970" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-90" yWindow="0" windowWidth="19380" windowHeight="20970" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -447,7 +447,7 @@
     <t>Group</t>
   </si>
   <si>
-    <t>UnitId[]</t>
+    <t>UnitId</t>
   </si>
 </sst>
 </file>
@@ -509,67 +509,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="7">
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="1">
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -1647,7 +1587,7 @@
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <conditionalFormatting sqref="A11:A16">
-    <cfRule type="duplicateValues" dxfId="6" priority="5"/>
+    <cfRule type="duplicateValues" dxfId="0" priority="5"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>